<commit_message>
Updated SPO1_mutant code and figures
</commit_message>
<xml_diff>
--- a/Optimal.entrap/Data/20260626_1522_cellsynchrony_github.xlsx
+++ b/Optimal.entrap/Data/20260626_1522_cellsynchrony_github.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joyobrien/GitHub/VirosporeQuant/Optimal.entrap/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joyobrien/GitHub/VirosporeQuant/Optimal.entrap/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3150FF0-D575-DC42-8DA0-530A1B3850D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A571E6-71A9-8D42-AEB3-569298F9675B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2120" yWindow="4100" windowWidth="27640" windowHeight="16940" xr2:uid="{6F350832-6EA5-FE43-AF0A-AA87720D692F}"/>
+    <workbookView xWindow="2120" yWindow="1580" windowWidth="27640" windowHeight="16940" xr2:uid="{6F350832-6EA5-FE43-AF0A-AA87720D692F}"/>
   </bookViews>
   <sheets>
     <sheet name="sync" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,8 +35,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={3701C47C-7832-F04A-BD15-A54B7DCF0EF9}</author>
+  </authors>
+  <commentList>
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{3701C47C-7832-F04A-BD15-A54B7DCF0EF9}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Need to correct for veg. cell count because non-heat treated CFU count is really total viable veg cells can be esimated as veg = non heat-treated cfu - heat treated cfu ml </t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Sample</t>
   </si>
@@ -125,17 +143,23 @@
     <t>T25R3</t>
   </si>
   <si>
-    <t>corr.veg.cells.ml</t>
-  </si>
-  <si>
     <t>total_cells</t>
+  </si>
+  <si>
+    <t>veg.cels.ml.corrected</t>
+  </si>
+  <si>
+    <t>veg.cells.ml.vol.corr</t>
+  </si>
+  <si>
+    <t>spores.ml.vol.corr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -148,6 +172,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -188,6 +218,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Joy O'Brien" id="{72184118-909C-3A43-B2F6-716029C829DD}" userId="S::jmo1056@usnh.edu::95b1195f-a313-4a17-a865-fbf58bce2244" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -505,12 +541,24 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="M1" dT="2026-09-02T18:47:13.12" personId="{72184118-909C-3A43-B2F6-716029C829DD}" id="{3701C47C-7832-F04A-BD15-A54B7DCF0EF9}">
+    <text xml:space="preserve">Need to correct for veg. cell count because non-heat treated CFU count is really total viable veg cells can be esimated as veg = non heat-treated cfu - heat treated cfu ml </text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5871077-6971-A548-B8A3-C81628DB73F7}">
-  <dimension ref="A1:M19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5871077-6971-A548-B8A3-C81628DB73F7}">
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="14" max="14" width="21.83203125" customWidth="1"/>
+    <col min="15" max="15" width="25.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -545,13 +593,19 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" t="s">
         <v>30</v>
       </c>
-      <c r="M1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -584,19 +638,27 @@
         <v>0.01</v>
       </c>
       <c r="K2" s="1">
-        <f>I2/(J2*G2)</f>
+        <f t="shared" ref="K2:K19" si="0">I2/(J2*G2)</f>
         <v>12000</v>
       </c>
       <c r="L2" s="1">
-        <f>H2+K2</f>
+        <f t="shared" ref="L2:L19" si="1">H2+K2</f>
         <v>90312000</v>
       </c>
       <c r="M2" s="1">
-        <f>L2-K2</f>
-        <v>90300000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+        <f>H2-K2</f>
+        <v>90288000</v>
+      </c>
+      <c r="N2" s="1">
+        <f>M2/8</f>
+        <v>11286000</v>
+      </c>
+      <c r="O2" s="1">
+        <f>K2/8</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -619,7 +681,7 @@
         <v>0.1</v>
       </c>
       <c r="H3" s="1">
-        <f t="shared" ref="H3:H19" si="0">E3/(F3*G3)</f>
+        <f t="shared" ref="H3:H19" si="2">E3/(F3*G3)</f>
         <v>136100000</v>
       </c>
       <c r="I3">
@@ -629,19 +691,27 @@
         <v>0.01</v>
       </c>
       <c r="K3" s="1">
-        <f>I3/(J3*G3)</f>
+        <f t="shared" si="0"/>
         <v>19000</v>
       </c>
       <c r="L3" s="1">
-        <f>H3+K3</f>
+        <f t="shared" si="1"/>
         <v>136119000</v>
       </c>
       <c r="M3" s="1">
-        <f t="shared" ref="M3:M19" si="1">L3-K3</f>
-        <v>136100000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" ref="M3:M19" si="3">H3-K3</f>
+        <v>136081000</v>
+      </c>
+      <c r="N3" s="1">
+        <f t="shared" ref="N3:N19" si="4">M3/8</f>
+        <v>17010125</v>
+      </c>
+      <c r="O3" s="1">
+        <f t="shared" ref="O3:O19" si="5">K3/8</f>
+        <v>2375</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -664,7 +734,7 @@
         <v>0.1</v>
       </c>
       <c r="H4" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>121999999.99999999</v>
       </c>
       <c r="I4">
@@ -674,19 +744,27 @@
         <v>0.01</v>
       </c>
       <c r="K4" s="1">
-        <f>I4/(J4*G4)</f>
+        <f t="shared" si="0"/>
         <v>9000</v>
       </c>
       <c r="L4" s="1">
-        <f>H4+K4</f>
+        <f t="shared" si="1"/>
         <v>122008999.99999999</v>
       </c>
       <c r="M4" s="1">
-        <f t="shared" si="1"/>
-        <v>121999999.99999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>121990999.99999999</v>
+      </c>
+      <c r="N4" s="1">
+        <f t="shared" si="4"/>
+        <v>15248874.999999998</v>
+      </c>
+      <c r="O4" s="1">
+        <f t="shared" si="5"/>
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -709,7 +787,7 @@
         <v>0.1</v>
       </c>
       <c r="H5" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10000000</v>
       </c>
       <c r="I5">
@@ -719,19 +797,27 @@
         <v>1E-4</v>
       </c>
       <c r="K5" s="1">
-        <f>I5/(J5*G5)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L5" s="1">
-        <f>H5+K5</f>
+        <f t="shared" si="1"/>
         <v>10000000</v>
       </c>
       <c r="M5" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>10000000</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N5" s="1">
+        <f t="shared" si="4"/>
+        <v>1250000</v>
+      </c>
+      <c r="O5" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -754,7 +840,7 @@
         <v>0.1</v>
       </c>
       <c r="H6" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>70000000</v>
       </c>
       <c r="I6">
@@ -764,19 +850,27 @@
         <v>1E-4</v>
       </c>
       <c r="K6" s="1">
-        <f>I6/(J6*G6)</f>
+        <f t="shared" si="0"/>
         <v>99999.999999999985</v>
       </c>
       <c r="L6" s="1">
-        <f>H6+K6</f>
+        <f t="shared" si="1"/>
         <v>70100000</v>
       </c>
       <c r="M6" s="1">
-        <f t="shared" si="1"/>
-        <v>70000000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>69900000</v>
+      </c>
+      <c r="N6" s="1">
+        <f t="shared" si="4"/>
+        <v>8737500</v>
+      </c>
+      <c r="O6" s="1">
+        <f t="shared" si="5"/>
+        <v>12499.999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -799,7 +893,7 @@
         <v>0.1</v>
       </c>
       <c r="H7" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>800000000</v>
       </c>
       <c r="I7">
@@ -809,19 +903,27 @@
         <v>1E-4</v>
       </c>
       <c r="K7" s="1">
-        <f>I7/(J7*G7)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L7" s="1">
-        <f>H7+K7</f>
+        <f t="shared" si="1"/>
         <v>800000000</v>
       </c>
       <c r="M7" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>800000000</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N7" s="1">
+        <f t="shared" si="4"/>
+        <v>100000000</v>
+      </c>
+      <c r="O7" s="1">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -844,7 +946,7 @@
         <v>0.1</v>
       </c>
       <c r="H8" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>530000000</v>
       </c>
       <c r="I8">
@@ -854,19 +956,27 @@
         <v>1E-4</v>
       </c>
       <c r="K8" s="1">
-        <f>I8/(J8*G8)</f>
+        <f t="shared" si="0"/>
         <v>5799999.9999999991</v>
       </c>
       <c r="L8" s="1">
-        <f>H8+K8</f>
+        <f t="shared" si="1"/>
         <v>535800000</v>
       </c>
       <c r="M8" s="1">
-        <f t="shared" si="1"/>
-        <v>530000000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>524200000</v>
+      </c>
+      <c r="N8" s="1">
+        <f t="shared" si="4"/>
+        <v>65525000</v>
+      </c>
+      <c r="O8" s="1">
+        <f t="shared" si="5"/>
+        <v>724999.99999999988</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -889,7 +999,7 @@
         <v>0.1</v>
       </c>
       <c r="H9" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>300000000</v>
       </c>
       <c r="I9">
@@ -899,19 +1009,27 @@
         <v>1E-4</v>
       </c>
       <c r="K9" s="1">
-        <f>I9/(J9*G9)</f>
+        <f t="shared" si="0"/>
         <v>6699999.9999999991</v>
       </c>
       <c r="L9" s="1">
-        <f>H9+K9</f>
+        <f t="shared" si="1"/>
         <v>306700000</v>
       </c>
       <c r="M9" s="1">
-        <f t="shared" si="1"/>
-        <v>300000000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>293300000</v>
+      </c>
+      <c r="N9" s="1">
+        <f t="shared" si="4"/>
+        <v>36662500</v>
+      </c>
+      <c r="O9" s="1">
+        <f t="shared" si="5"/>
+        <v>837499.99999999988</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -934,7 +1052,7 @@
         <v>0.1</v>
       </c>
       <c r="H10" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>660000000</v>
       </c>
       <c r="I10">
@@ -944,19 +1062,27 @@
         <v>1E-4</v>
       </c>
       <c r="K10" s="1">
-        <f>I10/(J10*G10)</f>
+        <f t="shared" si="0"/>
         <v>8299999.9999999991</v>
       </c>
       <c r="L10" s="1">
-        <f>H10+K10</f>
+        <f t="shared" si="1"/>
         <v>668300000</v>
       </c>
       <c r="M10" s="1">
-        <f t="shared" si="1"/>
-        <v>660000000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>651700000</v>
+      </c>
+      <c r="N10" s="1">
+        <f t="shared" si="4"/>
+        <v>81462500</v>
+      </c>
+      <c r="O10" s="1">
+        <f t="shared" si="5"/>
+        <v>1037499.9999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -979,7 +1105,7 @@
         <v>0.1</v>
       </c>
       <c r="H11" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>130000000</v>
       </c>
       <c r="I11">
@@ -989,19 +1115,27 @@
         <v>1E-4</v>
       </c>
       <c r="K11" s="1">
-        <f>I11/(J11*G11)</f>
+        <f t="shared" si="0"/>
         <v>26099999.999999996</v>
       </c>
       <c r="L11" s="1">
-        <f>H11+K11</f>
+        <f t="shared" si="1"/>
         <v>156100000</v>
       </c>
       <c r="M11" s="1">
-        <f t="shared" si="1"/>
-        <v>130000000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>103900000</v>
+      </c>
+      <c r="N11" s="1">
+        <f t="shared" si="4"/>
+        <v>12987500</v>
+      </c>
+      <c r="O11" s="1">
+        <f t="shared" si="5"/>
+        <v>3262499.9999999995</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1024,7 +1158,7 @@
         <v>0.1</v>
       </c>
       <c r="H12" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I12">
@@ -1034,19 +1168,24 @@
         <v>1E-4</v>
       </c>
       <c r="K12" s="1">
-        <f>I12/(J12*G12)</f>
+        <f t="shared" si="0"/>
         <v>50399999.999999993</v>
       </c>
       <c r="L12" s="1">
-        <f>H12+K12</f>
+        <f t="shared" si="1"/>
         <v>50399999.999999993</v>
       </c>
       <c r="M12" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>-50399999.999999993</v>
+      </c>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1">
+        <f t="shared" si="5"/>
+        <v>6299999.9999999991</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1069,7 +1208,7 @@
         <v>0.1</v>
       </c>
       <c r="H13" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>140000000</v>
       </c>
       <c r="I13">
@@ -1079,19 +1218,27 @@
         <v>1E-4</v>
       </c>
       <c r="K13" s="1">
-        <f>I13/(J13*G13)</f>
+        <f t="shared" si="0"/>
         <v>51399999.999999993</v>
       </c>
       <c r="L13" s="1">
-        <f>H13+K13</f>
+        <f t="shared" si="1"/>
         <v>191400000</v>
       </c>
       <c r="M13" s="1">
-        <f t="shared" si="1"/>
-        <v>140000000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>88600000</v>
+      </c>
+      <c r="N13" s="1">
+        <f t="shared" si="4"/>
+        <v>11075000</v>
+      </c>
+      <c r="O13" s="1">
+        <f t="shared" si="5"/>
+        <v>6424999.9999999991</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1114,7 +1261,7 @@
         <v>0.1</v>
       </c>
       <c r="H14" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>40900000</v>
       </c>
       <c r="I14">
@@ -1124,19 +1271,27 @@
         <v>1E-4</v>
       </c>
       <c r="K14" s="1">
-        <f>I14/(J14*G14)</f>
+        <f t="shared" si="0"/>
         <v>4099999.9999999995</v>
       </c>
       <c r="L14" s="1">
-        <f>H14+K14</f>
+        <f t="shared" si="1"/>
         <v>45000000</v>
       </c>
       <c r="M14" s="1">
-        <f t="shared" si="1"/>
-        <v>40900000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>36800000</v>
+      </c>
+      <c r="N14" s="1">
+        <f t="shared" si="4"/>
+        <v>4600000</v>
+      </c>
+      <c r="O14" s="1">
+        <f t="shared" si="5"/>
+        <v>512499.99999999994</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1159,7 +1314,7 @@
         <v>0.1</v>
       </c>
       <c r="H15" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>50399999.999999993</v>
       </c>
       <c r="I15">
@@ -1169,19 +1324,27 @@
         <v>1E-4</v>
       </c>
       <c r="K15" s="1">
-        <f>I15/(J15*G15)</f>
+        <f t="shared" si="0"/>
         <v>13799999.999999998</v>
       </c>
       <c r="L15" s="1">
-        <f>H15+K15</f>
+        <f t="shared" si="1"/>
         <v>64199999.999999993</v>
       </c>
       <c r="M15" s="1">
-        <f t="shared" si="1"/>
-        <v>50399999.999999993</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>36599999.999999993</v>
+      </c>
+      <c r="N15" s="1">
+        <f t="shared" si="4"/>
+        <v>4574999.9999999991</v>
+      </c>
+      <c r="O15" s="1">
+        <f t="shared" si="5"/>
+        <v>1724999.9999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1204,7 +1367,7 @@
         <v>0.1</v>
       </c>
       <c r="H16" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>136600000</v>
       </c>
       <c r="I16">
@@ -1214,19 +1377,27 @@
         <v>1E-4</v>
       </c>
       <c r="K16" s="1">
-        <f>I16/(J16*G16)</f>
+        <f t="shared" si="0"/>
         <v>33600000</v>
       </c>
       <c r="L16" s="1">
-        <f>H16+K16</f>
+        <f t="shared" si="1"/>
         <v>170200000</v>
       </c>
       <c r="M16" s="1">
-        <f t="shared" si="1"/>
-        <v>136600000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>103000000</v>
+      </c>
+      <c r="N16" s="1">
+        <f t="shared" si="4"/>
+        <v>12875000</v>
+      </c>
+      <c r="O16" s="1">
+        <f t="shared" si="5"/>
+        <v>4200000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1249,7 +1420,7 @@
         <v>0.1</v>
       </c>
       <c r="H17" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>114699999.99999999</v>
       </c>
       <c r="I17">
@@ -1259,19 +1430,26 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="K17" s="1">
-        <f>I17/(J17*G17)</f>
+        <f t="shared" si="0"/>
         <v>682999999.99999988</v>
       </c>
       <c r="L17" s="1">
-        <f>H17+K17</f>
+        <f t="shared" si="1"/>
         <v>797699999.99999988</v>
       </c>
       <c r="M17" s="1">
-        <f t="shared" si="1"/>
-        <v>114700000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>-568299999.99999988</v>
+      </c>
+      <c r="N17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <f t="shared" si="5"/>
+        <v>85374999.999999985</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1294,7 +1472,7 @@
         <v>0.1</v>
       </c>
       <c r="H18" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>50299999.999999993</v>
       </c>
       <c r="I18">
@@ -1304,19 +1482,26 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="K18" s="1">
-        <f>I18/(J18*G18)</f>
+        <f t="shared" si="0"/>
         <v>594999999.99999988</v>
       </c>
       <c r="L18" s="1">
-        <f>H18+K18</f>
+        <f t="shared" si="1"/>
         <v>645299999.99999988</v>
       </c>
       <c r="M18" s="1">
-        <f t="shared" si="1"/>
-        <v>50300000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+        <f t="shared" si="3"/>
+        <v>-544699999.99999988</v>
+      </c>
+      <c r="N18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
+        <f t="shared" si="5"/>
+        <v>74374999.999999985</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1339,7 +1524,7 @@
         <v>0.1</v>
       </c>
       <c r="H19" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>117799999.99999999</v>
       </c>
       <c r="I19">
@@ -1349,20 +1534,28 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="K19" s="1">
-        <f>I19/(J19*G19)</f>
+        <f t="shared" si="0"/>
         <v>836999999.99999988</v>
       </c>
       <c r="L19" s="1">
-        <f>H19+K19</f>
+        <f t="shared" si="1"/>
         <v>954799999.99999988</v>
       </c>
       <c r="M19" s="1">
-        <f t="shared" si="1"/>
-        <v>117800000</v>
+        <f t="shared" si="3"/>
+        <v>-719199999.99999988</v>
+      </c>
+      <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <f t="shared" si="5"/>
+        <v>104624999.99999999</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>